<commit_message>
Decouple auth-rbac services, add architecture docs and guides
Remove auth-rbac-service-backend and auth-rbac-service-frontend files
(moved to separate repositories). Update CLAUDE.md files to reflect
decoupled architecture. Add architecture diagrams, summary doc,
event mapping and notification rules guides.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bulk-upload-service/docs/test-order-delay.xlsx
+++ b/bulk-upload-service/docs/test-order-delay.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2995263-DAC5-4B92-B03D-0D9C6739A3B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F450FCB-3C98-4935-B8A2-0F3930907295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="order.delay" sheetId="1" r:id="rId1"/>
@@ -733,7 +733,7 @@
         <v>34</v>
       </c>
       <c r="G4">
-        <v>50240009954</v>
+        <v>50240009080</v>
       </c>
       <c r="H4" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
ui fixes and working
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bulk-upload-service/docs/test-order-delay.xlsx
+++ b/bulk-upload-service/docs/test-order-delay.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F450FCB-3C98-4935-B8A2-0F3930907295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA76D32B-E74E-4591-9F2D-F607648FDE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="order.delay" sheetId="1" r:id="rId1"/>
@@ -733,7 +733,7 @@
         <v>34</v>
       </c>
       <c r="G4">
-        <v>50240009080</v>
+        <v>50240009954</v>
       </c>
       <c r="H4" t="s">
         <v>35</v>

</xml_diff>